<commit_message>
feat: add back-to-back long weekend to Papá's plan (W7)
Adds the ultra-specific back-to-back (Sat 30 + Sun 16 on tired legs) at W7,
redistributing volume (52->54, within ramp cap) rather than spiking it, and
keeps the peak single long run at 37km. Best-practice long-run stimulus for
a 59km ultra without over-long single runs (masters recovery). Regenerated
plan_papa.md, Excel, and father_son doc.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Plan_Papa_UTT59.xlsx
+++ b/Plan_Papa_UTT59.xlsx
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>2100</v>
@@ -827,7 +827,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Peak build begins. Big vert week — descent legs get tested. Fuel every 40-45 min on the long run.</t>
+          <t>BACK-TO-BACK long weekend (Sat 30 + Sun 16 on tired legs) — the key ultra-specific session: simulates the cumulative fatigue of the race's back half. Easy pace; weekdays kept short to protect the weekend.</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="E45" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F45" s="8" t="n">
         <v>84</v>
@@ -2330,7 +2330,7 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F46" s="4" t="n">
         <v>630</v>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="E47" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F47" s="8" t="n">
         <v>84</v>
@@ -2427,33 +2427,33 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n">
+      <c r="A50" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="14" t="inlineStr">
         <is>
           <t>Domingo</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Carrera fácil</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F50" s="4" t="n">
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>Tirada larga — 16 km MEDIUM-LONG — back-to-back on tired legs</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="F50" s="14" t="n">
         <v>147</v>
       </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>120-130</t>
+      <c r="G50" s="14" t="inlineStr">
+        <is>
+          <t>120-135</t>
         </is>
       </c>
     </row>

</xml_diff>